<commit_message>
research: 3850·3969·1930·8095·6857·2884·3440·7818 2단계 브리프
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/jp/xlsx/3969.xlsx
+++ b/docs/data/jp/xlsx/3969.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="연간" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재무상태표" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="섹터 데이터" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'연간'!$3:$3</definedName>
@@ -21,14 +22,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0%;-0.0%;&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;;-0.0&quot;x&quot;;&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;년&quot;;-0.0&quot;년&quot;;&quot;-&quot;"/>
     <numFmt numFmtId="168" formatCode="0&quot;일&quot;;-0&quot;일&quot;;&quot;-&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0;\(#,##0.0\);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -126,11 +128,31 @@
     </font>
     <font>
       <name val="맑은 고딕"/>
+      <color rgb="FFFF0000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="FF808080"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -155,6 +177,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF808080"/>
       </patternFill>
     </fill>
     <fill>
@@ -201,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -345,7 +372,22 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9088,7 +9130,7 @@
     <row r="139">
       <c r="A139" s="20" t="inlineStr">
         <is>
-          <t>Payments Of Head Office Relocation Expenses Ope CF</t>
+          <t>본사 이전비용 지급액</t>
         </is>
       </c>
       <c r="D139" s="22" t="n">
@@ -9354,7 +9396,7 @@
     <row r="147">
       <c r="A147" s="20" t="inlineStr">
         <is>
-          <t>Purchase Of Golf Club Memberships Inv CF</t>
+          <t>골프 회원권 취득 지출</t>
         </is>
       </c>
       <c r="D147" s="22" t="n">
@@ -14190,6 +14232,706 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="52" t="inlineStr">
+        <is>
+          <t>에이트레드 섹터·사업 데이터</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>2단계 보고서를 만들 때 모은 자료 · 월차 · 출처는 맨 오른쪽</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="54" t="inlineStr">
+        <is>
+          <t>상반기 fy27</t>
+        </is>
+      </c>
+      <c r="B4" s="54" t="n"/>
+      <c r="C4" s="54" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="55" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="inlineStr">
+        <is>
+          <t>값</t>
+        </is>
+      </c>
+      <c r="C5" s="55" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="56" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B6" s="57" t="n">
+        <v>16.49</v>
+      </c>
+      <c r="C6" s="58" t="inlineStr">
+        <is>
+          <t>2단계 보고서 자료(회사 설명회 자료·공시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="56" t="inlineStr">
+        <is>
+          <t>매출 YoY</t>
+        </is>
+      </c>
+      <c r="B7" s="57" t="n">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="56" t="inlineStr">
+        <is>
+          <t>gp</t>
+        </is>
+      </c>
+      <c r="B8" s="57" t="n">
+        <v>10.61</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="56" t="inlineStr">
+        <is>
+          <t>sga</t>
+        </is>
+      </c>
+      <c r="B9" s="57" t="n">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="56" t="inlineStr">
+        <is>
+          <t>영업이익</t>
+        </is>
+      </c>
+      <c r="B10" s="57" t="n">
+        <v>5.57</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="56" t="inlineStr">
+        <is>
+          <t>영업이익 YoY</t>
+        </is>
+      </c>
+      <c r="B11" s="57" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>ordinary</t>
+        </is>
+      </c>
+      <c r="B12" s="57" t="n">
+        <v>5.74</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="56" t="inlineStr">
+        <is>
+          <t>ord YoY</t>
+        </is>
+      </c>
+      <c r="B13" s="57" t="n">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="56" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="B14" s="57" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="56" t="inlineStr">
+        <is>
+          <t>순이익 YoY</t>
+        </is>
+      </c>
+      <c r="B15" s="57" t="n">
+        <v>16.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="56" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="B16" s="57" t="n">
+        <v>50.22</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="54" t="inlineStr">
+        <is>
+          <t>상반기 fy27 · 계획 상반기</t>
+        </is>
+      </c>
+      <c r="B18" s="54" t="n"/>
+      <c r="C18" s="54" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="55" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B19" s="55" t="inlineStr">
+        <is>
+          <t>값</t>
+        </is>
+      </c>
+      <c r="C19" s="55" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="56" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B20" s="57" t="n">
+        <v>15.54</v>
+      </c>
+      <c r="C20" s="58" t="inlineStr">
+        <is>
+          <t>2단계 보고서 자료(회사 설명회 자료·공시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="56" t="inlineStr">
+        <is>
+          <t>영업이익</t>
+        </is>
+      </c>
+      <c r="B21" s="57" t="n">
+        <v>5.22</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="56" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="B22" s="57" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="54" t="inlineStr">
+        <is>
+          <t>2Q single calc</t>
+        </is>
+      </c>
+      <c r="B24" s="54" t="n"/>
+      <c r="C24" s="54" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="55" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B25" s="55" t="inlineStr">
+        <is>
+          <t>값</t>
+        </is>
+      </c>
+      <c r="C25" s="55" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="56" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B26" s="57" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="C26" s="58" t="inlineStr">
+        <is>
+          <t>2단계 보고서 자료(회사 설명회 자료·공시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="56" t="inlineStr">
+        <is>
+          <t>매출 YoY</t>
+        </is>
+      </c>
+      <c r="B27" s="57" t="n">
+        <v>21.3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="56" t="inlineStr">
+        <is>
+          <t>gp</t>
+        </is>
+      </c>
+      <c r="B28" s="57" t="n">
+        <v>5.65</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="56" t="inlineStr">
+        <is>
+          <t>매출총이익률</t>
+        </is>
+      </c>
+      <c r="B29" s="57" t="n">
+        <v>65.59999999999999</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="56" t="inlineStr">
+        <is>
+          <t>sga</t>
+        </is>
+      </c>
+      <c r="B30" s="57" t="n">
+        <v>2.62</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="56" t="inlineStr">
+        <is>
+          <t>영업이익</t>
+        </is>
+      </c>
+      <c r="B31" s="57" t="n">
+        <v>3.03</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="56" t="inlineStr">
+        <is>
+          <t>영업이익 YoY</t>
+        </is>
+      </c>
+      <c r="B32" s="57" t="n">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="56" t="inlineStr">
+        <is>
+          <t>영업이익률</t>
+        </is>
+      </c>
+      <c r="B33" s="57" t="n">
+        <v>35.2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="56" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="B34" s="57" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="56" t="inlineStr">
+        <is>
+          <t>순이익 YoY</t>
+        </is>
+      </c>
+      <c r="B35" s="57" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="56" t="inlineStr">
+        <is>
+          <t>cloud</t>
+        </is>
+      </c>
+      <c r="B36" s="57" t="n">
+        <v>4.66</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="56" t="inlineStr">
+        <is>
+          <t>cloud YoY</t>
+        </is>
+      </c>
+      <c r="B37" s="57" t="n">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="56" t="inlineStr">
+        <is>
+          <t>cloud QoQ add</t>
+        </is>
+      </c>
+      <c r="B38" s="57" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="56" t="inlineStr">
+        <is>
+          <t>aw</t>
+        </is>
+      </c>
+      <c r="B39" s="57" t="n">
+        <v>3.58</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="56" t="inlineStr">
+        <is>
+          <t>aw YoY</t>
+        </is>
+      </c>
+      <c r="B40" s="57" t="n">
+        <v>44.4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="56" t="inlineStr">
+        <is>
+          <t>xp</t>
+        </is>
+      </c>
+      <c r="B41" s="57" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="56" t="inlineStr">
+        <is>
+          <t>xp YoY</t>
+        </is>
+      </c>
+      <c r="B42" s="57" t="n">
+        <v>-23.9</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="54" t="inlineStr">
+        <is>
+          <t>2Q single calc · implied 계획 2q</t>
+        </is>
+      </c>
+      <c r="B44" s="54" t="n"/>
+      <c r="C44" s="54" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="55" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B45" s="55" t="inlineStr">
+        <is>
+          <t>값</t>
+        </is>
+      </c>
+      <c r="C45" s="55" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="56" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B46" s="57" t="n">
+        <v>7.66</v>
+      </c>
+      <c r="C46" s="58" t="inlineStr">
+        <is>
+          <t>2단계 보고서 자료(회사 설명회 자료·공시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="56" t="inlineStr">
+        <is>
+          <t>영업이익</t>
+        </is>
+      </c>
+      <c r="B47" s="57" t="n">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="54" t="inlineStr">
+        <is>
+          <t>가이던스 fy27</t>
+        </is>
+      </c>
+      <c r="B49" s="54" t="n"/>
+      <c r="C49" s="54" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="55" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B50" s="55" t="inlineStr">
+        <is>
+          <t>값</t>
+        </is>
+      </c>
+      <c r="C50" s="55" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="56" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B51" s="57" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="C51" s="58" t="inlineStr">
+        <is>
+          <t>2단계 보고서 자료(회사 설명회 자료·공시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="56" t="inlineStr">
+        <is>
+          <t>영업이익</t>
+        </is>
+      </c>
+      <c r="B52" s="57" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="56" t="inlineStr">
+        <is>
+          <t>ordinary</t>
+        </is>
+      </c>
+      <c r="B53" s="57" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="56" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="B54" s="57" t="n">
+        <v>7.83</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="56" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="B55" s="57" t="n">
+        <v>104.58</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="56" t="inlineStr">
+        <is>
+          <t>dps</t>
+        </is>
+      </c>
+      <c r="B56" s="59" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="54" t="inlineStr">
+        <is>
+          <t>가이던스 fy27 · 하반기 implied</t>
+        </is>
+      </c>
+      <c r="B58" s="54" t="n"/>
+      <c r="C58" s="54" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="55" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B59" s="55" t="inlineStr">
+        <is>
+          <t>값</t>
+        </is>
+      </c>
+      <c r="C59" s="55" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="56" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B60" s="57" t="n">
+        <v>16.11</v>
+      </c>
+      <c r="C60" s="58" t="inlineStr">
+        <is>
+          <t>2단계 보고서 자료(회사 설명회 자료·공시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="56" t="inlineStr">
+        <is>
+          <t>매출 YoY</t>
+        </is>
+      </c>
+      <c r="B61" s="57" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="56" t="inlineStr">
+        <is>
+          <t>영업이익</t>
+        </is>
+      </c>
+      <c r="B62" s="57" t="n">
+        <v>6.13</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="56" t="inlineStr">
+        <is>
+          <t>영업이익 YoY</t>
+        </is>
+      </c>
+      <c r="B63" s="57" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="54" t="inlineStr">
+        <is>
+          <t>preview · ours 2q</t>
+        </is>
+      </c>
+      <c r="B65" s="54" t="n"/>
+      <c r="C65" s="54" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="55" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B66" s="55" t="inlineStr">
+        <is>
+          <t>값</t>
+        </is>
+      </c>
+      <c r="C66" s="55" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="56" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B67" s="57" t="n">
+        <v>7.78</v>
+      </c>
+      <c r="C67" s="58" t="inlineStr">
+        <is>
+          <t>2단계 보고서 자료(회사 설명회 자료·공시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="56" t="inlineStr">
+        <is>
+          <t>영업이익</t>
+        </is>
+      </c>
+      <c r="B68" s="57" t="n">
+        <v>2.67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -14206,17 +14948,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="53" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>공시일</t>
         </is>
       </c>
-      <c r="B3" s="53" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>문서</t>
         </is>
       </c>
-      <c r="C3" s="53" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>

</xml_diff>